<commit_message>
Add Cowork reconciliation brief + rolling window, make pull payout-driven
- Rolling window: --days/--since/--until alongside --month.
- Payout-driven merge: one row per Stripe charge so each payout's lines
  tie to the exact bank deposit (even charges whose Luma sale predates
  the window); unmatched charges labelled instead of dropped.
- New Cowork brief (<out>_cowork_brief.md): one section per payout mapped
  to Xero Create fields (Who/What/Why/Event Name/Project Name/Tax Rate)
  with gross-income + Stripe-fee + Luma-fee split lines that total to the
  bank line. Only Stripe/Luma deposits listed; others left alone.
- event_map.json (Luma event name -> Xero Event Name tracking option),
  with .example; unmapped events flagged for manual pick.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Luma-Stripe-Reconcile/sample_reconciliation.xlsx
+++ b/Luma-Stripe-Reconcile/sample_reconciliation.xlsx
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -1046,7 +1046,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sales detail : one row per ticket sale, linked to its Stripe charge and payout.</t>
+          <t>Sales detail : one row per Stripe charge, linked to its Luma sale and payout.</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>each payout matches one transfer out of your Stripe clearing account.</t>
+          <t>each payout matches one received line in your bank feed.</t>
         </is>
       </c>
     </row>
@@ -1080,14 +1080,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UNMATCHED in a Stripe column = a Luma sale with no matching charge found</t>
+          <t>See the *_cowork_brief.md alongside this file for the per-payout Xero</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>(check email/amount, refunds, or a cross-month payout).</t>
+          <t>'Create' fields (Who / What / Why / Event Name / Project Name / Tax Rate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UNKNOWN (no Luma match) = a Stripe charge with no matching Luma sale found</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>(check email/amount, refunds, or pick the event manually).</t>
         </is>
       </c>
     </row>

</xml_diff>